<commit_message>
update to Excel only
</commit_message>
<xml_diff>
--- a/Scripts4Scripps.suite/Resources/ConsentForms.xlsx
+++ b/Scripts4Scripps.suite/Resources/ConsentForms.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ScriptRepositories\Scripps\Scripts4Scripps.suite\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01D6E04D-D45B-405E-96E7-CD5AC5EED6EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5E63ABE-58C9-4995-8EC8-067651DB4666}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{C864BDB0-4385-4BB3-84E1-4F66A64FF911}"/>
   </bookViews>
@@ -86,9 +86,6 @@
     <t>STANDARD ENDOSCOPIC RHYTIDECTOMY*</t>
   </si>
   <si>
-    <t>CHANGE FACIAL FEATURES</t>
-  </si>
-  <si>
     <t>ONE SYRINGE RESTYLANE*</t>
   </si>
   <si>
@@ -101,9 +98,6 @@
     <t>(A surgery to improve the cosmetic appearance of my _________by suctioning excess fat from under the surface of the skin.)</t>
   </si>
   <si>
-    <t>VASCULARIZED LYMPH NODE TRANSFER</t>
-  </si>
-  <si>
     <t>( ___________________ .)</t>
   </si>
   <si>
@@ -249,6 +243,12 @@
   </si>
   <si>
     <t>she|her</t>
+  </si>
+  <si>
+    <t>&lt;NONE&gt; CHANGE FACIAL FEATURES</t>
+  </si>
+  <si>
+    <t>&lt;NONE&gt; VASCULARIZED LYMPH NODE TRANSFER</t>
   </si>
 </sst>
 </file>
@@ -697,7 +697,7 @@
         <v>6</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -720,10 +720,10 @@
         <v>9</v>
       </c>
       <c r="D2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F2" t="s">
         <v>13</v>
@@ -737,19 +737,19 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F3" t="s">
         <v>14</v>
@@ -763,22 +763,22 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C4" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D4" t="s">
+        <v>66</v>
+      </c>
+      <c r="E4" t="s">
+        <v>58</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>68</v>
-      </c>
-      <c r="E4" t="s">
-        <v>60</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>15</v>
       </c>
       <c r="G4" t="s">
         <v>11</v>
@@ -789,25 +789,25 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C5" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D5" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G5" s="4" t="s">
         <v>16</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>17</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>12</v>
@@ -815,25 +815,25 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B6" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D6" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" s="4" t="s">
         <v>18</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>19</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>12</v>
@@ -841,25 +841,25 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D7" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E7" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>20</v>
+        <v>69</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>12</v>
@@ -867,25 +867,25 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B8" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D8" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E8" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F8" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="G8" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>12</v>
@@ -893,25 +893,25 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B9" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C9" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E9" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="F9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="G9" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>12</v>
@@ -919,25 +919,25 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B10" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C10" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D10" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E10" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F10" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G10" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>12</v>
@@ -945,25 +945,25 @@
     </row>
     <row r="11" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B11" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C11" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D11" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E11" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>12</v>

</xml_diff>